<commit_message>
Fixed first several mis-formatted cells
Last one changed Agelaius pheoniceus Syll Rep
</commit_message>
<xml_diff>
--- a/Source Data Process_CB/SupplementDataRefs_Update.xlsx
+++ b/Source Data Process_CB/SupplementDataRefs_Update.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kate/Desktop/CooperativeBreedingEvolution/Source Data Process_CB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6EAE43D9-A6CF-0041-BC60-A949470217DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9042A8D0-D882-1448-B9DC-1831B7C1E6CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9400" yWindow="460" windowWidth="29000" windowHeight="19380" xr2:uid="{1C1A7584-B053-4CE8-BA58-9497BFD2E86C}"/>
+    <workbookView xWindow="11620" yWindow="460" windowWidth="26780" windowHeight="19380" xr2:uid="{1C1A7584-B053-4CE8-BA58-9497BFD2E86C}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9481" uniqueCount="1972">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9484" uniqueCount="1975">
   <si>
     <t>BirdtreeFormat</t>
   </si>
@@ -6086,6 +6086,15 @@
   </si>
   <si>
     <t>References cited in Data tab</t>
+  </si>
+  <si>
+    <t>10-20</t>
+  </si>
+  <si>
+    <t>5-25</t>
+  </si>
+  <si>
+    <t>7-30</t>
   </si>
 </sst>
 </file>
@@ -7305,8 +7314,8 @@
       <c r="I16" s="3">
         <v>15</v>
       </c>
-      <c r="J16" s="3">
-        <v>43393</v>
+      <c r="J16" s="3" t="s">
+        <v>1972</v>
       </c>
       <c r="K16" s="3" t="s">
         <v>58</v>
@@ -7632,8 +7641,8 @@
       <c r="I21" s="3">
         <v>15</v>
       </c>
-      <c r="J21" s="3">
-        <v>43245</v>
+      <c r="J21" s="3" t="s">
+        <v>1973</v>
       </c>
       <c r="K21" s="3" t="s">
         <v>81</v>
@@ -7832,8 +7841,8 @@
       <c r="I25" s="3">
         <v>18.5</v>
       </c>
-      <c r="J25" s="3">
-        <v>43311</v>
+      <c r="J25" s="3" t="s">
+        <v>1974</v>
       </c>
       <c r="K25" s="3" t="s">
         <v>89</v>

</xml_diff>

<commit_message>
Fixed misformatted Sylls/song source data
</commit_message>
<xml_diff>
--- a/Source Data Process_CB/SupplementDataRefs_Update.xlsx
+++ b/Source Data Process_CB/SupplementDataRefs_Update.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kate/Desktop/CooperativeBreedingEvolution/Source Data Process_CB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{866B85F1-8C1D-7E45-9374-3B414B4AD53E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA2AB13E-4A31-9F46-8D1F-6DFCAC887D21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14740" yWindow="700" windowWidth="26780" windowHeight="19380" xr2:uid="{1C1A7584-B053-4CE8-BA58-9497BFD2E86C}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9487" uniqueCount="1978">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9491" uniqueCount="1982">
   <si>
     <t>BirdtreeFormat</t>
   </si>
@@ -6104,6 +6104,18 @@
   </si>
   <si>
     <t>9-20</t>
+  </si>
+  <si>
+    <t>1-3</t>
+  </si>
+  <si>
+    <t>2-3</t>
+  </si>
+  <si>
+    <t>7-10</t>
+  </si>
+  <si>
+    <t>3-5</t>
   </si>
 </sst>
 </file>
@@ -11394,8 +11406,8 @@
       <c r="L95" s="3">
         <v>2</v>
       </c>
-      <c r="M95" s="3">
-        <v>43103</v>
+      <c r="M95" s="3" t="s">
+        <v>1978</v>
       </c>
       <c r="N95" s="3" t="s">
         <v>93</v>
@@ -20357,8 +20369,8 @@
       <c r="L270" s="3">
         <v>2.5</v>
       </c>
-      <c r="M270" s="3">
-        <v>43134</v>
+      <c r="M270" s="3" t="s">
+        <v>1979</v>
       </c>
       <c r="N270" s="3" t="s">
         <v>93</v>
@@ -41117,8 +41129,8 @@
       <c r="L682" s="3">
         <v>8.5</v>
       </c>
-      <c r="M682" s="3">
-        <v>43291</v>
+      <c r="M682" s="3" t="s">
+        <v>1980</v>
       </c>
       <c r="N682" s="3" t="s">
         <v>93</v>
@@ -41744,8 +41756,8 @@
       <c r="L695" s="3">
         <v>4</v>
       </c>
-      <c r="M695" s="3">
-        <v>43164</v>
+      <c r="M695" s="3" t="s">
+        <v>1981</v>
       </c>
       <c r="N695" s="3" t="s">
         <v>93</v>

</xml_diff>

<commit_message>
added missing source data for Interval for Fringilla coelebs
</commit_message>
<xml_diff>
--- a/Source Data Process_CB/SupplementDataRefs_Update.xlsx
+++ b/Source Data Process_CB/SupplementDataRefs_Update.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kate/Desktop/CooperativeBreedingEvolution/Source Data Process_CB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA2AB13E-4A31-9F46-8D1F-6DFCAC887D21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B644A2F-1CC1-A24A-9265-22461B86303F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14740" yWindow="700" windowWidth="26780" windowHeight="19380" xr2:uid="{1C1A7584-B053-4CE8-BA58-9497BFD2E86C}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9491" uniqueCount="1982">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9493" uniqueCount="1984">
   <si>
     <t>BirdtreeFormat</t>
   </si>
@@ -6116,6 +6116,12 @@
   </si>
   <si>
     <t>3-5</t>
+  </si>
+  <si>
+    <t>8.09; 8.07</t>
+  </si>
+  <si>
+    <t>8.08</t>
   </si>
 </sst>
 </file>
@@ -22938,10 +22944,12 @@
       <c r="T321" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="U321" s="3">
-        <v>8.09</v>
-      </c>
-      <c r="V321" s="3"/>
+      <c r="U321" s="3" t="s">
+        <v>1983</v>
+      </c>
+      <c r="V321" s="3" t="s">
+        <v>1982</v>
+      </c>
       <c r="W321" s="3" t="s">
         <v>555</v>
       </c>

</xml_diff>

<commit_message>
Update Syllable repertoire entry for Turdus philomelos
Urban 95% CI: 343.58-422.85 (mean of these two values considered population mean)
Forest 95% CI: 276.05–335.72 (mean of these two values considered population mean)
Mean of two population means is overall species value (344.6); Forest population mean is species minimum (305.9), Urban population mean is species maximum (383.2)

Deoniziak K, Osiejuk TS. Habitat-related differences in song structure and complexity in a songbird with a large repertoire. BMC Ecol. 2019 Sep 18;19(1):40. doi: 10.1186/s12898-019-0255-7. PMID: 31533798; PMCID: PMC6749692.
</commit_message>
<xml_diff>
--- a/Source Data Process_CB/SupplementDataRefs_Update.xlsx
+++ b/Source Data Process_CB/SupplementDataRefs_Update.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10509"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10711"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kate/Desktop/CooperativeBreedingEvolution/Source Data Process_CB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B644A2F-1CC1-A24A-9265-22461B86303F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD526A2E-B22E-3945-AFE7-87D123FA4863}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14740" yWindow="700" windowWidth="26780" windowHeight="19380" xr2:uid="{1C1A7584-B053-4CE8-BA58-9497BFD2E86C}"/>
+    <workbookView xWindow="11620" yWindow="700" windowWidth="26780" windowHeight="19380" xr2:uid="{1C1A7584-B053-4CE8-BA58-9497BFD2E86C}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9493" uniqueCount="1984">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9496" uniqueCount="1988">
   <si>
     <t>BirdtreeFormat</t>
   </si>
@@ -6123,12 +6123,24 @@
   <si>
     <t>8.08</t>
   </si>
+  <si>
+    <t>Deoniziak and Osiejuk (2019)</t>
+  </si>
+  <si>
+    <t>Two populations (Forest, Urban): 305.9, 383.2</t>
+  </si>
+  <si>
+    <t>344.6</t>
+  </si>
+  <si>
+    <t>Deoniziak K, Osiejuk TS. Habitat-related differences in song structure and complexity in a songbird with a large repertoire. BMC Ecol. 2019 Sep 18;19(1):40. doi: 10.1186/s12898-019-0255-7. PMID: 31533798; PMCID: PMC6749692.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -6154,6 +6166,13 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF212121"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -6191,7 +6210,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
@@ -6206,6 +6225,7 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -50317,10 +50337,14 @@
       <c r="G861" s="3"/>
       <c r="H861" s="3"/>
       <c r="I861" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="J861" s="3"/>
-      <c r="K861" s="3"/>
+        <v>1986</v>
+      </c>
+      <c r="J861" s="3" t="s">
+        <v>1985</v>
+      </c>
+      <c r="K861" s="3" t="s">
+        <v>1984</v>
+      </c>
       <c r="L861" s="3">
         <v>9</v>
       </c>
@@ -53053,7 +53077,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3B1421C-CED3-49E2-A372-9BE4C43E3345}">
-  <dimension ref="A1:A188"/>
+  <dimension ref="A1:A189"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
@@ -53267,732 +53291,737 @@
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A43" s="2" t="s">
-        <v>1824</v>
+      <c r="A43" s="6" t="s">
+        <v>1987</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>1825</v>
+        <v>1824</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>1826</v>
+        <v>1825</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>1827</v>
+        <v>1826</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
-        <v>1828</v>
+        <v>1827</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
-        <v>1829</v>
+        <v>1828</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
-        <v>1830</v>
+        <v>1829</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
-        <v>1831</v>
+        <v>1830</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
-        <v>1832</v>
+        <v>1831</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>1833</v>
+        <v>1832</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
-        <v>1834</v>
+        <v>1833</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>1835</v>
+        <v>1834</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
-        <v>1836</v>
+        <v>1835</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
-        <v>1837</v>
+        <v>1836</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
-        <v>1838</v>
+        <v>1837</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
-        <v>1839</v>
+        <v>1838</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
-        <v>1840</v>
+        <v>1839</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
-        <v>1841</v>
+        <v>1840</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
-        <v>1842</v>
+        <v>1841</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
-        <v>1844</v>
+        <v>1843</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
-        <v>1845</v>
+        <v>1844</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
-        <v>1846</v>
+        <v>1845</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
-        <v>1847</v>
+        <v>1846</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
-        <v>1848</v>
+        <v>1847</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
-        <v>1849</v>
+        <v>1848</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
-        <v>1850</v>
+        <v>1849</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
-        <v>1851</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
-        <v>1852</v>
+        <v>1851</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
-        <v>1853</v>
+        <v>1852</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
-        <v>1854</v>
+        <v>1853</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
-        <v>1855</v>
+        <v>1854</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
-        <v>1856</v>
+        <v>1855</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A76" s="2" t="s">
-        <v>1857</v>
+        <v>1856</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
-        <v>1858</v>
+        <v>1857</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
-        <v>1859</v>
+        <v>1858</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A79" s="2" t="s">
-        <v>1860</v>
+        <v>1859</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
-        <v>1861</v>
+        <v>1860</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A81" s="2" t="s">
-        <v>1862</v>
+        <v>1861</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
-        <v>1863</v>
+        <v>1862</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A83" s="2" t="s">
-        <v>1864</v>
+        <v>1863</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A84" s="2" t="s">
-        <v>1865</v>
+        <v>1864</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A85" s="2" t="s">
-        <v>1866</v>
+        <v>1865</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
-        <v>1867</v>
+        <v>1866</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
-        <v>1868</v>
+        <v>1867</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
-        <v>1869</v>
+        <v>1868</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
-        <v>1870</v>
+        <v>1869</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A90" s="2" t="s">
-        <v>1871</v>
+        <v>1870</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
-        <v>1872</v>
+        <v>1871</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A92" s="2" t="s">
-        <v>1873</v>
+        <v>1872</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A93" s="2" t="s">
-        <v>1874</v>
+        <v>1873</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
-        <v>1875</v>
+        <v>1874</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A95" s="2" t="s">
-        <v>1876</v>
+        <v>1875</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
-        <v>1877</v>
+        <v>1876</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
-        <v>1878</v>
+        <v>1877</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
-        <v>1879</v>
+        <v>1878</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
-        <v>1880</v>
+        <v>1879</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A100" s="2" t="s">
-        <v>1881</v>
+        <v>1880</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A101" s="2" t="s">
-        <v>1882</v>
+        <v>1881</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A102" s="2" t="s">
-        <v>1883</v>
+        <v>1882</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A103" s="2" t="s">
-        <v>1884</v>
+        <v>1883</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A104" s="2" t="s">
-        <v>1885</v>
+        <v>1884</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A105" s="2" t="s">
-        <v>1886</v>
+        <v>1885</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A106" s="2" t="s">
-        <v>1887</v>
+        <v>1886</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A107" s="2" t="s">
-        <v>1888</v>
+        <v>1887</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A108" s="2" t="s">
-        <v>1889</v>
+        <v>1888</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A109" s="2" t="s">
-        <v>1890</v>
+        <v>1889</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A110" s="2" t="s">
-        <v>1891</v>
+        <v>1890</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A111" s="2" t="s">
-        <v>1892</v>
+        <v>1891</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A112" s="2" t="s">
-        <v>1893</v>
+        <v>1892</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A113" s="2" t="s">
-        <v>1894</v>
+        <v>1893</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A114" s="2" t="s">
-        <v>1895</v>
+        <v>1894</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A115" s="2" t="s">
-        <v>1896</v>
+        <v>1895</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A116" s="2" t="s">
-        <v>1897</v>
+        <v>1896</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A117" s="2" t="s">
-        <v>1898</v>
+        <v>1897</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A118" s="2" t="s">
-        <v>1899</v>
+        <v>1898</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A119" s="2" t="s">
-        <v>1900</v>
+        <v>1899</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A120" s="2" t="s">
-        <v>1901</v>
+        <v>1900</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A121" s="2" t="s">
-        <v>1902</v>
+        <v>1901</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A122" s="2" t="s">
-        <v>1903</v>
+        <v>1902</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A123" s="2" t="s">
-        <v>1904</v>
+        <v>1903</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A124" s="2" t="s">
-        <v>1905</v>
+        <v>1904</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A125" s="2" t="s">
+        <v>1905</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A126" s="2" t="s">
         <v>1906</v>
       </c>
     </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A126" s="1" t="s">
+    <row r="127" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A127" s="1" t="s">
         <v>1907</v>
-      </c>
-    </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A127" s="2" t="s">
-        <v>1908</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A128" s="2" t="s">
+        <v>1908</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A129" s="2" t="s">
         <v>1909</v>
       </c>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A129" s="1" t="s">
+    <row r="130" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A130" s="1" t="s">
         <v>1910</v>
-      </c>
-    </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A130" s="2" t="s">
-        <v>1911</v>
       </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A131" s="2" t="s">
-        <v>1912</v>
+        <v>1911</v>
       </c>
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A132" s="2" t="s">
-        <v>1913</v>
+        <v>1912</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A133" s="2" t="s">
-        <v>1914</v>
+        <v>1913</v>
       </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A134" s="2" t="s">
-        <v>1915</v>
+        <v>1914</v>
       </c>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A135" s="2" t="s">
-        <v>1916</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A136" s="2" t="s">
-        <v>1917</v>
+        <v>1916</v>
       </c>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A137" s="2" t="s">
-        <v>1918</v>
+        <v>1917</v>
       </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A138" s="2" t="s">
-        <v>1919</v>
+        <v>1918</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A139" s="2" t="s">
-        <v>1920</v>
+        <v>1919</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A140" s="2" t="s">
-        <v>1921</v>
+        <v>1920</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A141" s="2" t="s">
-        <v>1922</v>
+        <v>1921</v>
       </c>
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A142" s="2" t="s">
-        <v>1923</v>
+        <v>1922</v>
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A143" s="2" t="s">
-        <v>1924</v>
+        <v>1923</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A144" s="2" t="s">
+        <v>1924</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A145" s="2" t="s">
         <v>1925</v>
       </c>
     </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A145" s="1" t="s">
+    <row r="146" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A146" s="1" t="s">
         <v>1926</v>
-      </c>
-    </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A146" s="2" t="s">
-        <v>1927</v>
       </c>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A147" s="2" t="s">
-        <v>1928</v>
+        <v>1927</v>
       </c>
     </row>
     <row r="148" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A148" s="2" t="s">
+        <v>1928</v>
+      </c>
+    </row>
+    <row r="149" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A149" s="2" t="s">
         <v>1929</v>
       </c>
     </row>
-    <row r="149" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A149" s="1" t="s">
+    <row r="150" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A150" s="1" t="s">
         <v>1930</v>
-      </c>
-    </row>
-    <row r="150" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A150" s="2" t="s">
-        <v>1931</v>
       </c>
     </row>
     <row r="151" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A151" s="2" t="s">
-        <v>1932</v>
+        <v>1931</v>
       </c>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A152" s="2" t="s">
-        <v>1933</v>
+        <v>1932</v>
       </c>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A153" s="2" t="s">
-        <v>1934</v>
+        <v>1933</v>
       </c>
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A154" s="2" t="s">
-        <v>1935</v>
+        <v>1934</v>
       </c>
     </row>
     <row r="155" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A155" s="2" t="s">
-        <v>1936</v>
+        <v>1935</v>
       </c>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A156" s="2" t="s">
-        <v>1937</v>
+        <v>1936</v>
       </c>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A157" s="2" t="s">
-        <v>1938</v>
+        <v>1937</v>
       </c>
     </row>
     <row r="158" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A158" s="2" t="s">
-        <v>1939</v>
+        <v>1938</v>
       </c>
     </row>
     <row r="159" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A159" s="2" t="s">
-        <v>1940</v>
+        <v>1939</v>
       </c>
     </row>
     <row r="160" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A160" s="2" t="s">
-        <v>1941</v>
+        <v>1940</v>
       </c>
     </row>
     <row r="161" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A161" s="2" t="s">
-        <v>1942</v>
+        <v>1941</v>
       </c>
     </row>
     <row r="162" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A162" s="2" t="s">
-        <v>1943</v>
+        <v>1942</v>
       </c>
     </row>
     <row r="163" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A163" s="2" t="s">
-        <v>1944</v>
+        <v>1943</v>
       </c>
     </row>
     <row r="164" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A164" s="2" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
     </row>
     <row r="165" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A165" s="2" t="s">
-        <v>1946</v>
+        <v>1945</v>
       </c>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A166" s="2" t="s">
-        <v>1947</v>
+        <v>1946</v>
       </c>
     </row>
     <row r="167" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A167" s="2" t="s">
+        <v>1947</v>
+      </c>
+    </row>
+    <row r="168" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A168" s="2" t="s">
         <v>1948</v>
-      </c>
-    </row>
-    <row r="168" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A168" s="1" t="s">
-        <v>1949</v>
       </c>
     </row>
     <row r="169" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A169" s="1" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="170" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A170" s="1" t="s">
         <v>1950</v>
-      </c>
-    </row>
-    <row r="170" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A170" s="2" t="s">
-        <v>1951</v>
       </c>
     </row>
     <row r="171" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A171" s="2" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
     </row>
     <row r="172" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A172" s="2" t="s">
-        <v>1953</v>
+        <v>1952</v>
       </c>
     </row>
     <row r="173" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A173" s="2" t="s">
-        <v>1954</v>
+        <v>1953</v>
       </c>
     </row>
     <row r="174" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A174" s="2" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
     </row>
     <row r="175" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A175" s="2" t="s">
-        <v>1956</v>
+        <v>1955</v>
       </c>
     </row>
     <row r="176" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A176" s="2" t="s">
-        <v>1957</v>
+        <v>1956</v>
       </c>
     </row>
     <row r="177" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A177" s="2" t="s">
-        <v>1958</v>
+        <v>1957</v>
       </c>
     </row>
     <row r="178" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A178" s="2" t="s">
-        <v>1959</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="179" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A179" s="2" t="s">
-        <v>1960</v>
+        <v>1959</v>
       </c>
     </row>
     <row r="180" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A180" s="2" t="s">
-        <v>1961</v>
+        <v>1960</v>
       </c>
     </row>
     <row r="181" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A181" s="2" t="s">
-        <v>1962</v>
+        <v>1961</v>
       </c>
     </row>
     <row r="182" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A182" s="2" t="s">
-        <v>1963</v>
+        <v>1962</v>
       </c>
     </row>
     <row r="183" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A183" s="2" t="s">
-        <v>1964</v>
+        <v>1963</v>
       </c>
     </row>
     <row r="184" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A184" s="2" t="s">
-        <v>1965</v>
+        <v>1964</v>
       </c>
     </row>
     <row r="185" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A185" s="2" t="s">
-        <v>1966</v>
+        <v>1965</v>
       </c>
     </row>
     <row r="186" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A186" s="2" t="s">
-        <v>1967</v>
+        <v>1966</v>
       </c>
     </row>
     <row r="187" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A187" s="2" t="s">
-        <v>1968</v>
+        <v>1967</v>
       </c>
     </row>
     <row r="188" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A188" s="2" t="s">
+        <v>1968</v>
+      </c>
+    </row>
+    <row r="189" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A189" s="2" t="s">
         <v>1969</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Syllable repertoire data, update species-level song values for Hirundo rustica
Added value syllable repertoire = 27.6 from:
Wilkins MR, Shizuka D, Joseph MB, Hubbard JK, Safran RJ. Multimodal signalling in the North American barn swallow: a phenotype network approach. Proc Biol Sci. 2015 Oct 7;282(1816):20151574. doi: 10.1098/rspb.2015.1574. PMID: 26423842; PMCID: PMC4614773.

Also re-calculated Rate and Continuity values for Hirundo rustica based on new min, max, and mean values from Garamszegi et al (2006)
</commit_message>
<xml_diff>
--- a/Source Data Process_CB/SupplementDataRefs_Update.xlsx
+++ b/Source Data Process_CB/SupplementDataRefs_Update.xlsx
@@ -8,25 +8,34 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kate/Desktop/CooperativeBreedingEvolution/Source Data Process_CB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70A78EA8-DEFB-7346-AE69-2854EDDC5B41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F29C97C7-80B2-054E-9263-466DE7B7849F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11200" yWindow="460" windowWidth="26780" windowHeight="19380" activeTab="1" xr2:uid="{1C1A7584-B053-4CE8-BA58-9497BFD2E86C}"/>
+    <workbookView xWindow="1180" yWindow="460" windowWidth="26780" windowHeight="19380" xr2:uid="{1C1A7584-B053-4CE8-BA58-9497BFD2E86C}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
     <sheet name="References" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="179017"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9497" uniqueCount="1990">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9501" uniqueCount="1994">
   <si>
     <t>BirdtreeFormat</t>
   </si>
@@ -6121,18 +6130,12 @@
     <t>Deoniziak K, Osiejuk TS. Habitat-related differences in song structure and complexity in a songbird with a large repertoire. BMC Ecol. 2019 Sep 18;19(1):40. doi: 10.1186/s12898-019-0255-7. PMID: 31533798; PMCID: PMC6749692.</t>
   </si>
   <si>
-    <t>20; 22.9</t>
-  </si>
-  <si>
     <t>12; 16.9; 19.8; 17.8</t>
   </si>
   <si>
     <t>DeVoogd et al (1993); Soma and Garamszegi (2011); Garamszegi and Moller (2004); Garamszegi et al (2006)</t>
   </si>
   <si>
-    <t>Galeotti et al (1997) via Moore, et al (2011); Garamszegi et al (2006)</t>
-  </si>
-  <si>
     <t>4.01; 6; 4.75</t>
   </si>
   <si>
@@ -6140,6 +6143,24 @@
   </si>
   <si>
     <t>Garamszegi LZ, Hegyi G, Heylen D, Ninni P, de Lope F, Eens M, Møller AP. The design of complex sexual traits in male barn swallows: associations between signal attributes. J Evol Biol. 2006 Nov;19(6):2052-66. doi: 10.1111/j.1420-9101.2006.01135.x. PMID: 17040402.</t>
+  </si>
+  <si>
+    <t>20; 22.9; 27.6</t>
+  </si>
+  <si>
+    <t>Galeotti et al (1997) via Moore, et al (2011); Garamszegi et al (2006); Wilkins et al (2015)</t>
+  </si>
+  <si>
+    <t>Wilkins MR, Shizuka D, Joseph MB, Hubbard JK, Safran RJ. Multimodal signalling in the North American barn swallow: a phenotype network approach. Proc Biol Sci. 2015 Oct 7;282(1816):20151574. doi: 10.1098/rspb.2015.1574. PMID: 26423842; PMCID: PMC4614773.</t>
+  </si>
+  <si>
+    <t>22.9</t>
+  </si>
+  <si>
+    <t>17.4</t>
+  </si>
+  <si>
+    <t>4.75</t>
   </si>
 </sst>
 </file>
@@ -24318,23 +24339,23 @@
       <c r="H349" s="3" t="s">
         <v>1674</v>
       </c>
-      <c r="I349" s="3">
-        <v>20.100000000000001</v>
+      <c r="I349" s="3" t="s">
+        <v>1991</v>
       </c>
       <c r="J349" s="3" t="s">
+        <v>1988</v>
+      </c>
+      <c r="K349" s="3" t="s">
+        <v>1989</v>
+      </c>
+      <c r="L349" s="3" t="s">
+        <v>1992</v>
+      </c>
+      <c r="M349" s="3" t="s">
         <v>1983</v>
       </c>
-      <c r="K349" s="3" t="s">
-        <v>1986</v>
-      </c>
-      <c r="L349" s="3">
-        <v>16.899999999999999</v>
-      </c>
-      <c r="M349" s="3" t="s">
+      <c r="N349" s="3" t="s">
         <v>1984</v>
-      </c>
-      <c r="N349" s="3" t="s">
-        <v>1985</v>
       </c>
       <c r="O349" s="3">
         <v>56</v>
@@ -24345,14 +24366,14 @@
       <c r="Q349" s="3" t="s">
         <v>592</v>
       </c>
-      <c r="R349" s="3">
-        <v>5.0049999999999999</v>
+      <c r="R349" s="3" t="s">
+        <v>1993</v>
       </c>
       <c r="S349" s="3" t="s">
-        <v>1987</v>
+        <v>1985</v>
       </c>
       <c r="T349" s="3" t="s">
-        <v>1988</v>
+        <v>1986</v>
       </c>
       <c r="U349" s="3">
         <v>3.0249999999999999</v>
@@ -53083,7 +53104,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3B1421C-CED3-49E2-A372-9BE4C43E3345}">
-  <dimension ref="A1:A190"/>
+  <dimension ref="A1:A191"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
@@ -53393,7 +53414,7 @@
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A62" s="6" t="s">
-        <v>1989</v>
+        <v>1987</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.2">
@@ -54022,17 +54043,22 @@
       </c>
     </row>
     <row r="188" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A188" s="2" t="s">
-        <v>1962</v>
+      <c r="A188" s="6" t="s">
+        <v>1990</v>
       </c>
     </row>
     <row r="189" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A189" s="2" t="s">
-        <v>1963</v>
+        <v>1962</v>
       </c>
     </row>
     <row r="190" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A190" s="2" t="s">
+        <v>1963</v>
+      </c>
+    </row>
+    <row r="191" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A191" s="2" t="s">
         <v>1964</v>
       </c>
     </row>

</xml_diff>